<commit_message>
minor edits to tables and figures
</commit_message>
<xml_diff>
--- a/Models/Model Outputs/TraitModels_Formatted.xlsx
+++ b/Models/Model Outputs/TraitModels_Formatted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sarahjennings/Desktop/MAPS-Phenology-Project/Models/Model Outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAE3662-B0A8-D943-98BE-2324ACA2D690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344B6D45-51EA-064D-BED7-090DFEE57522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1420" yWindow="500" windowWidth="26840" windowHeight="15060" xr2:uid="{23DB0BCD-A074-5F44-9464-C3A450BBDB70}"/>
   </bookViews>
@@ -831,19 +831,19 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1260,13 +1260,13 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="10" t="s">
         <v>11</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -1278,17 +1278,17 @@
       <c r="F2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="11">
+      <c r="G2" s="13">
         <v>0</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="13">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="9"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="10"/>
       <c r="D3" s="4" t="s">
         <v>0</v>
       </c>
@@ -1298,13 +1298,13 @@
       <c r="F3" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="12"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="9"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="10"/>
       <c r="D4" s="4" t="s">
         <v>14</v>
       </c>
@@ -1314,13 +1314,13 @@
       <c r="F4" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="9" t="s">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -1332,17 +1332,17 @@
       <c r="F5" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="10">
         <v>0</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="9"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="10"/>
       <c r="D6" s="4" t="s">
         <v>0</v>
       </c>
@@ -1352,13 +1352,13 @@
       <c r="F6" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="9"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="4" t="s">
         <v>14</v>
       </c>
@@ -1368,8 +1368,8 @@
       <c r="F7" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
     </row>
     <row r="8" spans="1:8" ht="4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4"/>
@@ -1382,13 +1382,13 @@
       <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -1400,17 +1400,17 @@
       <c r="F9" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="10">
         <v>0</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="9"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="10"/>
       <c r="D10" s="4" t="s">
         <v>1</v>
       </c>
@@ -1420,13 +1420,13 @@
       <c r="F10" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="9"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="10"/>
       <c r="D11" s="4" t="s">
         <v>14</v>
       </c>
@@ -1436,13 +1436,13 @@
       <c r="F11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="9" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -1454,17 +1454,17 @@
       <c r="F12" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="10">
         <v>0</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="9"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="10"/>
       <c r="D13" s="4" t="s">
         <v>1</v>
       </c>
@@ -1474,13 +1474,13 @@
       <c r="F13" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="9"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="10"/>
       <c r="D14" s="4" t="s">
         <v>14</v>
       </c>
@@ -1490,8 +1490,8 @@
       <c r="F14" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" spans="1:8" ht="4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4"/>
@@ -1504,13 +1504,13 @@
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>11</v>
       </c>
       <c r="D16" s="4" t="s">
@@ -1522,17 +1522,17 @@
       <c r="F16" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="10">
         <v>0</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="9"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="10"/>
       <c r="D17" s="4" t="s">
         <v>17</v>
       </c>
@@ -1542,13 +1542,13 @@
       <c r="F17" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="9"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="10"/>
       <c r="D18" s="4" t="s">
         <v>14</v>
       </c>
@@ -1558,13 +1558,13 @@
       <c r="F18" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="9" t="s">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="4" t="s">
@@ -1576,17 +1576,17 @@
       <c r="F19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="10">
         <v>0</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="9"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="10"/>
       <c r="D20" s="4" t="s">
         <v>17</v>
       </c>
@@ -1596,13 +1596,13 @@
       <c r="F20" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="9"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="10"/>
       <c r="D21" s="4" t="s">
         <v>14</v>
       </c>
@@ -1612,8 +1612,8 @@
       <c r="F21" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4"/>
@@ -1626,13 +1626,13 @@
       <c r="H22" s="6"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="10" t="s">
         <v>11</v>
       </c>
       <c r="D23" s="4" t="s">
@@ -1644,17 +1644,17 @@
       <c r="F23" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="10">
         <v>0</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="9"/>
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="10"/>
       <c r="D24" s="4" t="s">
         <v>17</v>
       </c>
@@ -1664,13 +1664,13 @@
       <c r="F24" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="9"/>
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="10"/>
       <c r="D25" s="4" t="s">
         <v>14</v>
       </c>
@@ -1680,13 +1680,13 @@
       <c r="F25" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="9" t="s">
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D26" s="4" t="s">
@@ -1698,17 +1698,17 @@
       <c r="F26" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="10">
         <v>0</v>
       </c>
-      <c r="H26" s="9">
+      <c r="H26" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="9"/>
+      <c r="A27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="10"/>
       <c r="D27" s="4" t="s">
         <v>17</v>
       </c>
@@ -1718,13 +1718,13 @@
       <c r="F27" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="9"/>
+      <c r="A28" s="9"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="10"/>
       <c r="D28" s="4" t="s">
         <v>14</v>
       </c>
@@ -1734,8 +1734,8 @@
       <c r="F28" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
@@ -1748,13 +1748,13 @@
       <c r="H29" s="6"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="10" t="s">
         <v>11</v>
       </c>
       <c r="D30" s="4" t="s">
@@ -1766,17 +1766,17 @@
       <c r="F30" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G30" s="9">
+      <c r="G30" s="10">
         <v>0</v>
       </c>
-      <c r="H30" s="9">
-        <v>20</v>
+      <c r="H30" s="10">
+        <v>18</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="9"/>
+      <c r="A31" s="9"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="10"/>
       <c r="D31" s="4" t="s">
         <v>2</v>
       </c>
@@ -1786,13 +1786,13 @@
       <c r="F31" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="12"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="9"/>
+      <c r="A32" s="9"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="10"/>
       <c r="D32" s="4" t="s">
         <v>14</v>
       </c>
@@ -1802,13 +1802,13 @@
       <c r="F32" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G32" s="9"/>
-      <c r="H32" s="9"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="12"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="9" t="s">
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D33" s="4" t="s">
@@ -1820,17 +1820,17 @@
       <c r="F33" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G33" s="9">
+      <c r="G33" s="10">
         <v>0</v>
       </c>
-      <c r="H33" s="9">
-        <v>20</v>
+      <c r="H33" s="10">
+        <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="12"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="9"/>
+      <c r="A34" s="9"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="10"/>
       <c r="D34" s="4" t="s">
         <v>2</v>
       </c>
@@ -1840,13 +1840,13 @@
       <c r="F34" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="13"/>
-      <c r="B35" s="13"/>
-      <c r="C35" s="10"/>
+      <c r="A35" s="12"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="11"/>
       <c r="D35" s="7" t="s">
         <v>14</v>
       </c>
@@ -1856,31 +1856,15 @@
       <c r="F35" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="B2:B7"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="B9:B14"/>
-    <mergeCell ref="C9:C11"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="C33:C35"/>
-    <mergeCell ref="A16:A21"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="B23:B28"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="B30:B35"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="H23:H25"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="H30:H32"/>
+    <mergeCell ref="H33:H35"/>
     <mergeCell ref="G23:G25"/>
     <mergeCell ref="G26:G28"/>
     <mergeCell ref="G30:G32"/>
@@ -1897,10 +1881,26 @@
     <mergeCell ref="G16:G18"/>
     <mergeCell ref="G19:G21"/>
     <mergeCell ref="H19:H21"/>
-    <mergeCell ref="H23:H25"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="H30:H32"/>
-    <mergeCell ref="H33:H35"/>
+    <mergeCell ref="C33:C35"/>
+    <mergeCell ref="A16:A21"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="B23:B28"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="B30:B35"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="A9:A14"/>
+    <mergeCell ref="B9:B14"/>
+    <mergeCell ref="C9:C11"/>
+    <mergeCell ref="C12:C14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>